<commit_message>
Remove substitution cardinality from medication profile 3ebe7870b066881a10b325ea3f4c924bdbe82e86
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-request.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-request.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-12T15:16:17+00:00</t>
+    <t>2026-08-13T08:08:00+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -17733,7 +17733,7 @@
       </c>
       <c r="E127" s="2"/>
       <c r="F127" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G127" t="s" s="2">
         <v>91</v>

</xml_diff>

<commit_message>
Refactor dosageInstruction constraints in FSH profile
Removed specific constraints on dosageInstruction fields for doseRange and rateRange. eb5149ae12698dec37dab17d971df8cd7406a7db
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-request.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-request.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5995" uniqueCount="923">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5556" uniqueCount="884">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-13T09:15:12+00:00</t>
+    <t>2026-08-13T09:41:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2196,68 +2196,14 @@
     <t>Dose à administrer</t>
   </si>
   <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x]:doseRange.id</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x].id</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x]:doseRange.extension</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x].extension</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x]:doseRange.low</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x].low</t>
+    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x]:doseQuantity</t>
+  </si>
+  <si>
+    <t>doseQuantity</t>
   </si>
   <si>
     <t xml:space="preserve">Quantity {SimpleQuantity|4.0.1}
 </t>
-  </si>
-  <si>
-    <t>Low limit</t>
-  </si>
-  <si>
-    <t>The low limit. The boundary is inclusive.</t>
-  </si>
-  <si>
-    <t>If the low element is missing, the low boundary is not known.</t>
-  </si>
-  <si>
-    <t>Range.low</t>
-  </si>
-  <si>
-    <t>NR.1</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x]:doseRange.high</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x].high</t>
-  </si>
-  <si>
-    <t>High limit</t>
-  </si>
-  <si>
-    <t>The high limit. The boundary is inclusive.</t>
-  </si>
-  <si>
-    <t>If the high element is missing, the high boundary is not known.</t>
-  </si>
-  <si>
-    <t>Range.high</t>
-  </si>
-  <si>
-    <t>NR.2</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.dose[x]:doseQuantity</t>
-  </si>
-  <si>
-    <t>doseQuantity</t>
   </si>
   <si>
     <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x]</t>
@@ -2299,30 +2245,6 @@
     <t>Rythme d'administration</t>
   </si>
   <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x]:rateRange.id</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x].id</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x]:rateRange.extension</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x].extension</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x]:rateRange.low</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x].low</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x]:rateRange.high</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.doseAndRate.rate[x].high</t>
-  </si>
-  <si>
     <t>MedicationRequest.dosageInstruction.maxDosePerPeriod</t>
   </si>
   <si>
@@ -2349,46 +2271,6 @@
   </si>
   <si>
     <t>RXO-23, RXE-19</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.maxDosePerPeriod.id</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.maxDosePerPeriod.extension</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.maxDosePerPeriod.numerator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantity
-</t>
-  </si>
-  <si>
-    <t>Numerator value</t>
-  </si>
-  <si>
-    <t>The value of the numerator.</t>
-  </si>
-  <si>
-    <t>Ratio.numerator</t>
-  </si>
-  <si>
-    <t>.numerator</t>
-  </si>
-  <si>
-    <t>MedicationRequest.dosageInstruction.maxDosePerPeriod.denominator</t>
-  </si>
-  <si>
-    <t>Denominator value</t>
-  </si>
-  <si>
-    <t>The value of the denominator.</t>
-  </si>
-  <si>
-    <t>Ratio.denominator</t>
-  </si>
-  <si>
-    <t>.denominator</t>
   </si>
   <si>
     <t>MedicationRequest.dosageInstruction.maxDosePerAdministration</t>
@@ -3189,7 +3071,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO162"/>
+  <dimension ref="A1:AO150"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="69.60546875" customWidth="true" bestFit="true"/>
@@ -9070,7 +8952,7 @@
         <v>80</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>82</v>
@@ -11049,7 +10931,7 @@
         <v>80</v>
       </c>
       <c r="G68" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H68" t="s" s="2">
         <v>82</v>
@@ -15821,9 +15703,11 @@
         <v>700</v>
       </c>
       <c r="B109" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="C109" t="s" s="2">
         <v>701</v>
       </c>
-      <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
         <v>82</v>
       </c>
@@ -15841,19 +15725,23 @@
         <v>82</v>
       </c>
       <c r="J109" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K109" t="s" s="2">
-        <v>168</v>
+        <v>702</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>169</v>
+        <v>689</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="N109" s="2"/>
-      <c r="O109" s="2"/>
+        <v>690</v>
+      </c>
+      <c r="N109" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="O109" t="s" s="2">
+        <v>692</v>
+      </c>
       <c r="P109" t="s" s="2">
         <v>82</v>
       </c>
@@ -15901,7 +15789,7 @@
         <v>82</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>171</v>
+        <v>694</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>80</v>
@@ -15913,7 +15801,7 @@
         <v>82</v>
       </c>
       <c r="AJ109" t="s" s="2">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="AK109" t="s" s="2">
         <v>82</v>
@@ -15922,32 +15810,32 @@
         <v>82</v>
       </c>
       <c r="AM109" t="s" s="2">
-        <v>172</v>
+        <v>670</v>
       </c>
       <c r="AN109" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO109" t="s" s="2">
-        <v>82</v>
+        <v>695</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B110" t="s" s="2">
         <v>703</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
-        <v>216</v>
+        <v>82</v>
       </c>
       <c r="E110" s="2"/>
       <c r="F110" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G110" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H110" t="s" s="2">
         <v>82</v>
@@ -15956,21 +15844,23 @@
         <v>82</v>
       </c>
       <c r="J110" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K110" t="s" s="2">
-        <v>136</v>
+        <v>704</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>421</v>
+        <v>705</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>422</v>
+        <v>706</v>
       </c>
       <c r="N110" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="O110" s="2"/>
+        <v>707</v>
+      </c>
+      <c r="O110" t="s" s="2">
+        <v>708</v>
+      </c>
       <c r="P110" t="s" s="2">
         <v>82</v>
       </c>
@@ -16006,11 +15896,9 @@
         <v>82</v>
       </c>
       <c r="AB110" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AC110" t="s" s="2">
-        <v>175</v>
-      </c>
+        <v>518</v>
+      </c>
+      <c r="AC110" s="2"/>
       <c r="AD110" t="s" s="2">
         <v>82</v>
       </c>
@@ -16018,19 +15906,19 @@
         <v>140</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>176</v>
+        <v>709</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH110" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI110" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ110" t="s" s="2">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="AK110" t="s" s="2">
         <v>82</v>
@@ -16039,29 +15927,31 @@
         <v>82</v>
       </c>
       <c r="AM110" t="s" s="2">
-        <v>172</v>
+        <v>710</v>
       </c>
       <c r="AN110" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO110" t="s" s="2">
-        <v>82</v>
+        <v>711</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>705</v>
-      </c>
-      <c r="C111" s="2"/>
+        <v>703</v>
+      </c>
+      <c r="C111" t="s" s="2">
+        <v>713</v>
+      </c>
       <c r="D111" t="s" s="2">
         <v>82</v>
       </c>
       <c r="E111" s="2"/>
       <c r="F111" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G111" t="s" s="2">
         <v>91</v>
@@ -16076,18 +15966,20 @@
         <v>92</v>
       </c>
       <c r="K111" t="s" s="2">
+        <v>698</v>
+      </c>
+      <c r="L111" t="s" s="2">
+        <v>714</v>
+      </c>
+      <c r="M111" t="s" s="2">
         <v>706</v>
       </c>
-      <c r="L111" t="s" s="2">
+      <c r="N111" t="s" s="2">
         <v>707</v>
       </c>
-      <c r="M111" t="s" s="2">
+      <c r="O111" t="s" s="2">
         <v>708</v>
       </c>
-      <c r="N111" t="s" s="2">
-        <v>709</v>
-      </c>
-      <c r="O111" s="2"/>
       <c r="P111" t="s" s="2">
         <v>82</v>
       </c>
@@ -16135,7 +16027,7 @@
         <v>82</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>80</v>
@@ -16156,7 +16048,7 @@
         <v>82</v>
       </c>
       <c r="AM111" t="s" s="2">
-        <v>536</v>
+        <v>710</v>
       </c>
       <c r="AN111" t="s" s="2">
         <v>82</v>
@@ -16167,10 +16059,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -16178,7 +16070,7 @@
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G112" t="s" s="2">
         <v>91</v>
@@ -16193,18 +16085,20 @@
         <v>92</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>706</v>
+        <v>716</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="N112" t="s" s="2">
-        <v>716</v>
-      </c>
-      <c r="O112" s="2"/>
+        <v>719</v>
+      </c>
+      <c r="O112" t="s" s="2">
+        <v>720</v>
+      </c>
       <c r="P112" t="s" s="2">
         <v>82</v>
       </c>
@@ -16252,7 +16146,7 @@
         <v>82</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>80</v>
@@ -16273,25 +16167,23 @@
         <v>82</v>
       </c>
       <c r="AM112" t="s" s="2">
-        <v>545</v>
+        <v>722</v>
       </c>
       <c r="AN112" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO112" t="s" s="2">
-        <v>718</v>
+        <v>723</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>687</v>
-      </c>
-      <c r="C113" t="s" s="2">
-        <v>720</v>
-      </c>
+        <v>724</v>
+      </c>
+      <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
         <v>82</v>
       </c>
@@ -16312,19 +16204,19 @@
         <v>92</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>689</v>
+        <v>725</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>690</v>
+        <v>726</v>
       </c>
       <c r="N113" t="s" s="2">
-        <v>691</v>
+        <v>727</v>
       </c>
       <c r="O113" t="s" s="2">
-        <v>692</v>
+        <v>728</v>
       </c>
       <c r="P113" t="s" s="2">
         <v>82</v>
@@ -16373,7 +16265,7 @@
         <v>82</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>694</v>
+        <v>729</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>80</v>
@@ -16394,21 +16286,21 @@
         <v>82</v>
       </c>
       <c r="AM113" t="s" s="2">
-        <v>670</v>
+        <v>730</v>
       </c>
       <c r="AN113" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO113" t="s" s="2">
-        <v>695</v>
+        <v>82</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -16431,19 +16323,17 @@
         <v>92</v>
       </c>
       <c r="K114" t="s" s="2">
-        <v>722</v>
+        <v>702</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>723</v>
+        <v>732</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>724</v>
-      </c>
-      <c r="N114" t="s" s="2">
-        <v>725</v>
-      </c>
+        <v>733</v>
+      </c>
+      <c r="N114" s="2"/>
       <c r="O114" t="s" s="2">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="P114" t="s" s="2">
         <v>82</v>
@@ -16480,17 +16370,19 @@
         <v>82</v>
       </c>
       <c r="AB114" t="s" s="2">
-        <v>518</v>
-      </c>
-      <c r="AC114" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="AC114" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="AD114" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE114" t="s" s="2">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>80</v>
@@ -16511,25 +16403,23 @@
         <v>82</v>
       </c>
       <c r="AM114" t="s" s="2">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="AN114" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO114" t="s" s="2">
-        <v>729</v>
+        <v>82</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>721</v>
-      </c>
-      <c r="C115" t="s" s="2">
-        <v>731</v>
-      </c>
+        <v>736</v>
+      </c>
+      <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
         <v>82</v>
       </c>
@@ -16547,23 +16437,19 @@
         <v>82</v>
       </c>
       <c r="J115" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K115" t="s" s="2">
-        <v>698</v>
+        <v>737</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>724</v>
-      </c>
-      <c r="N115" t="s" s="2">
-        <v>725</v>
-      </c>
-      <c r="O115" t="s" s="2">
-        <v>726</v>
-      </c>
+        <v>739</v>
+      </c>
+      <c r="N115" s="2"/>
+      <c r="O115" s="2"/>
       <c r="P115" t="s" s="2">
         <v>82</v>
       </c>
@@ -16611,7 +16497,7 @@
         <v>82</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>727</v>
+        <v>736</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>80</v>
@@ -16629,24 +16515,24 @@
         <v>82</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>82</v>
+        <v>740</v>
       </c>
       <c r="AM115" t="s" s="2">
-        <v>728</v>
+        <v>741</v>
       </c>
       <c r="AN115" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO115" t="s" s="2">
-        <v>729</v>
+        <v>82</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>733</v>
+        <v>742</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -16758,14 +16644,14 @@
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
-        <v>216</v>
+        <v>82</v>
       </c>
       <c r="E117" s="2"/>
       <c r="F117" t="s" s="2">
@@ -16787,14 +16673,12 @@
         <v>136</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>421</v>
+        <v>137</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="N117" t="s" s="2">
-        <v>219</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="N117" s="2"/>
       <c r="O117" s="2"/>
       <c r="P117" t="s" s="2">
         <v>82</v>
@@ -16833,9 +16717,7 @@
       <c r="AB117" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="AC117" t="s" s="2">
-        <v>175</v>
-      </c>
+      <c r="AC117" s="2"/>
       <c r="AD117" t="s" s="2">
         <v>82</v>
       </c>
@@ -16864,7 +16746,7 @@
         <v>82</v>
       </c>
       <c r="AM117" t="s" s="2">
-        <v>172</v>
+        <v>82</v>
       </c>
       <c r="AN117" t="s" s="2">
         <v>82</v>
@@ -16875,18 +16757,20 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>738</v>
-      </c>
-      <c r="C118" s="2"/>
+        <v>743</v>
+      </c>
+      <c r="C118" t="s" s="2">
+        <v>745</v>
+      </c>
       <c r="D118" t="s" s="2">
         <v>82</v>
       </c>
       <c r="E118" s="2"/>
       <c r="F118" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G118" t="s" s="2">
         <v>91</v>
@@ -16898,20 +16782,18 @@
         <v>82</v>
       </c>
       <c r="J118" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>706</v>
+        <v>746</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>707</v>
+        <v>747</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>708</v>
-      </c>
-      <c r="N118" t="s" s="2">
-        <v>709</v>
-      </c>
+        <v>748</v>
+      </c>
+      <c r="N118" s="2"/>
       <c r="O118" s="2"/>
       <c r="P118" t="s" s="2">
         <v>82</v>
@@ -16960,19 +16842,19 @@
         <v>82</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>710</v>
+        <v>176</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH118" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI118" t="s" s="2">
-        <v>82</v>
+        <v>149</v>
       </c>
       <c r="AJ118" t="s" s="2">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="AK118" t="s" s="2">
         <v>82</v>
@@ -16981,29 +16863,31 @@
         <v>82</v>
       </c>
       <c r="AM118" t="s" s="2">
-        <v>536</v>
+        <v>82</v>
       </c>
       <c r="AN118" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO118" t="s" s="2">
-        <v>711</v>
+        <v>82</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>739</v>
+        <v>749</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>740</v>
-      </c>
-      <c r="C119" s="2"/>
+        <v>743</v>
+      </c>
+      <c r="C119" t="s" s="2">
+        <v>750</v>
+      </c>
       <c r="D119" t="s" s="2">
         <v>82</v>
       </c>
       <c r="E119" s="2"/>
       <c r="F119" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G119" t="s" s="2">
         <v>91</v>
@@ -17015,19 +16899,19 @@
         <v>82</v>
       </c>
       <c r="J119" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K119" t="s" s="2">
-        <v>706</v>
+        <v>751</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>714</v>
+        <v>752</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>715</v>
+        <v>753</v>
       </c>
       <c r="N119" t="s" s="2">
-        <v>716</v>
+        <v>754</v>
       </c>
       <c r="O119" s="2"/>
       <c r="P119" t="s" s="2">
@@ -17077,19 +16961,19 @@
         <v>82</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>717</v>
+        <v>176</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH119" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI119" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ119" t="s" s="2">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="AK119" t="s" s="2">
         <v>82</v>
@@ -17098,21 +16982,21 @@
         <v>82</v>
       </c>
       <c r="AM119" t="s" s="2">
-        <v>545</v>
+        <v>82</v>
       </c>
       <c r="AN119" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO119" t="s" s="2">
-        <v>718</v>
+        <v>82</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s" s="2">
-        <v>741</v>
+        <v>755</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>741</v>
+        <v>756</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -17132,23 +17016,19 @@
         <v>82</v>
       </c>
       <c r="J120" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K120" t="s" s="2">
-        <v>742</v>
+        <v>168</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>743</v>
+        <v>169</v>
       </c>
       <c r="M120" t="s" s="2">
-        <v>744</v>
-      </c>
-      <c r="N120" t="s" s="2">
-        <v>745</v>
-      </c>
-      <c r="O120" t="s" s="2">
-        <v>746</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="N120" s="2"/>
+      <c r="O120" s="2"/>
       <c r="P120" t="s" s="2">
         <v>82</v>
       </c>
@@ -17196,7 +17076,7 @@
         <v>82</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>747</v>
+        <v>171</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>80</v>
@@ -17208,7 +17088,7 @@
         <v>82</v>
       </c>
       <c r="AJ120" t="s" s="2">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="AK120" t="s" s="2">
         <v>82</v>
@@ -17217,21 +17097,21 @@
         <v>82</v>
       </c>
       <c r="AM120" t="s" s="2">
-        <v>748</v>
+        <v>172</v>
       </c>
       <c r="AN120" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO120" t="s" s="2">
-        <v>749</v>
+        <v>82</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>750</v>
+        <v>758</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -17242,7 +17122,7 @@
         <v>80</v>
       </c>
       <c r="G121" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H121" t="s" s="2">
         <v>82</v>
@@ -17254,13 +17134,13 @@
         <v>82</v>
       </c>
       <c r="K121" t="s" s="2">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="L121" t="s" s="2">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="M121" t="s" s="2">
-        <v>170</v>
+        <v>138</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
@@ -17299,31 +17179,31 @@
         <v>82</v>
       </c>
       <c r="AB121" t="s" s="2">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="AC121" t="s" s="2">
-        <v>82</v>
+        <v>175</v>
       </c>
       <c r="AD121" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE121" t="s" s="2">
-        <v>82</v>
+        <v>140</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH121" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI121" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ121" t="s" s="2">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="AK121" t="s" s="2">
         <v>82</v>
@@ -17332,7 +17212,7 @@
         <v>82</v>
       </c>
       <c r="AM121" t="s" s="2">
-        <v>172</v>
+        <v>82</v>
       </c>
       <c r="AN121" t="s" s="2">
         <v>82</v>
@@ -17343,21 +17223,21 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>751</v>
+        <v>760</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
-        <v>216</v>
+        <v>82</v>
       </c>
       <c r="E122" s="2"/>
       <c r="F122" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G122" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H122" t="s" s="2">
         <v>82</v>
@@ -17369,16 +17249,16 @@
         <v>82</v>
       </c>
       <c r="K122" t="s" s="2">
-        <v>136</v>
+        <v>105</v>
       </c>
       <c r="L122" t="s" s="2">
-        <v>421</v>
+        <v>185</v>
       </c>
       <c r="M122" t="s" s="2">
-        <v>422</v>
+        <v>186</v>
       </c>
       <c r="N122" t="s" s="2">
-        <v>219</v>
+        <v>187</v>
       </c>
       <c r="O122" s="2"/>
       <c r="P122" t="s" s="2">
@@ -17386,7 +17266,7 @@
       </c>
       <c r="Q122" s="2"/>
       <c r="R122" t="s" s="2">
-        <v>82</v>
+        <v>761</v>
       </c>
       <c r="S122" t="s" s="2">
         <v>82</v>
@@ -17416,31 +17296,31 @@
         <v>82</v>
       </c>
       <c r="AB122" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AC122" t="s" s="2">
-        <v>175</v>
+        <v>82</v>
       </c>
       <c r="AD122" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE122" t="s" s="2">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="AG122" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AH122" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI122" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ122" t="s" s="2">
-        <v>142</v>
+        <v>82</v>
       </c>
       <c r="AK122" t="s" s="2">
         <v>82</v>
@@ -17449,7 +17329,7 @@
         <v>82</v>
       </c>
       <c r="AM122" t="s" s="2">
-        <v>172</v>
+        <v>134</v>
       </c>
       <c r="AN122" t="s" s="2">
         <v>82</v>
@@ -17460,10 +17340,10 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>752</v>
+        <v>762</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>752</v>
+        <v>763</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -17483,16 +17363,16 @@
         <v>82</v>
       </c>
       <c r="J123" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K123" t="s" s="2">
-        <v>753</v>
+        <v>413</v>
       </c>
       <c r="L123" t="s" s="2">
-        <v>754</v>
+        <v>764</v>
       </c>
       <c r="M123" t="s" s="2">
-        <v>755</v>
+        <v>765</v>
       </c>
       <c r="N123" s="2"/>
       <c r="O123" s="2"/>
@@ -17543,7 +17423,7 @@
         <v>82</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>756</v>
+        <v>194</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>80</v>
@@ -17564,7 +17444,7 @@
         <v>82</v>
       </c>
       <c r="AM123" t="s" s="2">
-        <v>757</v>
+        <v>134</v>
       </c>
       <c r="AN123" t="s" s="2">
         <v>82</v>
@@ -17575,42 +17455,46 @@
     </row>
     <row r="124">
       <c r="A124" t="s" s="2">
-        <v>758</v>
+        <v>766</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>758</v>
+        <v>766</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
-        <v>82</v>
+        <v>451</v>
       </c>
       <c r="E124" s="2"/>
       <c r="F124" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G124" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H124" t="s" s="2">
         <v>82</v>
       </c>
       <c r="I124" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="J124" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K124" t="s" s="2">
-        <v>753</v>
+        <v>136</v>
       </c>
       <c r="L124" t="s" s="2">
-        <v>759</v>
+        <v>452</v>
       </c>
       <c r="M124" t="s" s="2">
-        <v>760</v>
-      </c>
-      <c r="N124" s="2"/>
-      <c r="O124" s="2"/>
+        <v>453</v>
+      </c>
+      <c r="N124" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="O124" t="s" s="2">
+        <v>220</v>
+      </c>
       <c r="P124" t="s" s="2">
         <v>82</v>
       </c>
@@ -17658,19 +17542,19 @@
         <v>82</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>761</v>
+        <v>454</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH124" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI124" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ124" t="s" s="2">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="AK124" t="s" s="2">
         <v>82</v>
@@ -17679,7 +17563,7 @@
         <v>82</v>
       </c>
       <c r="AM124" t="s" s="2">
-        <v>762</v>
+        <v>134</v>
       </c>
       <c r="AN124" t="s" s="2">
         <v>82</v>
@@ -17690,10 +17574,10 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -17713,23 +17597,21 @@
         <v>82</v>
       </c>
       <c r="J125" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K125" t="s" s="2">
-        <v>706</v>
+        <v>737</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="M125" t="s" s="2">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="N125" t="s" s="2">
-        <v>766</v>
-      </c>
-      <c r="O125" t="s" s="2">
-        <v>767</v>
-      </c>
+        <v>770</v>
+      </c>
+      <c r="O125" s="2"/>
       <c r="P125" t="s" s="2">
         <v>82</v>
       </c>
@@ -17777,7 +17659,7 @@
         <v>82</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>80</v>
@@ -17798,7 +17680,7 @@
         <v>82</v>
       </c>
       <c r="AM125" t="s" s="2">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="AN125" t="s" s="2">
         <v>82</v>
@@ -17809,10 +17691,10 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -17832,21 +17714,19 @@
         <v>82</v>
       </c>
       <c r="J126" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K126" t="s" s="2">
-        <v>706</v>
+        <v>168</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>771</v>
+        <v>169</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>772</v>
+        <v>170</v>
       </c>
       <c r="N126" s="2"/>
-      <c r="O126" t="s" s="2">
-        <v>773</v>
-      </c>
+      <c r="O126" s="2"/>
       <c r="P126" t="s" s="2">
         <v>82</v>
       </c>
@@ -17894,7 +17774,7 @@
         <v>82</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>774</v>
+        <v>171</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>80</v>
@@ -17906,7 +17786,7 @@
         <v>82</v>
       </c>
       <c r="AJ126" t="s" s="2">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="AK126" t="s" s="2">
         <v>82</v>
@@ -17915,7 +17795,7 @@
         <v>82</v>
       </c>
       <c r="AM126" t="s" s="2">
-        <v>769</v>
+        <v>172</v>
       </c>
       <c r="AN126" t="s" s="2">
         <v>82</v>
@@ -17926,21 +17806,21 @@
     </row>
     <row r="127">
       <c r="A127" t="s" s="2">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
-        <v>82</v>
+        <v>216</v>
       </c>
       <c r="E127" s="2"/>
       <c r="F127" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G127" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H127" t="s" s="2">
         <v>82</v>
@@ -17952,15 +17832,17 @@
         <v>82</v>
       </c>
       <c r="K127" t="s" s="2">
-        <v>776</v>
+        <v>136</v>
       </c>
       <c r="L127" t="s" s="2">
-        <v>777</v>
+        <v>421</v>
       </c>
       <c r="M127" t="s" s="2">
-        <v>778</v>
-      </c>
-      <c r="N127" s="2"/>
+        <v>422</v>
+      </c>
+      <c r="N127" t="s" s="2">
+        <v>219</v>
+      </c>
       <c r="O127" s="2"/>
       <c r="P127" t="s" s="2">
         <v>82</v>
@@ -18009,28 +17891,28 @@
         <v>82</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>775</v>
+        <v>176</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH127" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI127" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ127" t="s" s="2">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="AK127" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL127" t="s" s="2">
-        <v>779</v>
+        <v>82</v>
       </c>
       <c r="AM127" t="s" s="2">
-        <v>780</v>
+        <v>172</v>
       </c>
       <c r="AN127" t="s" s="2">
         <v>82</v>
@@ -18041,42 +17923,46 @@
     </row>
     <row r="128">
       <c r="A128" t="s" s="2">
-        <v>781</v>
+        <v>774</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>781</v>
+        <v>774</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
-        <v>82</v>
+        <v>451</v>
       </c>
       <c r="E128" s="2"/>
       <c r="F128" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G128" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H128" t="s" s="2">
         <v>82</v>
       </c>
       <c r="I128" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="J128" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K128" t="s" s="2">
-        <v>168</v>
+        <v>136</v>
       </c>
       <c r="L128" t="s" s="2">
-        <v>169</v>
+        <v>452</v>
       </c>
       <c r="M128" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="N128" s="2"/>
-      <c r="O128" s="2"/>
+        <v>453</v>
+      </c>
+      <c r="N128" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="O128" t="s" s="2">
+        <v>220</v>
+      </c>
       <c r="P128" t="s" s="2">
         <v>82</v>
       </c>
@@ -18124,19 +18010,19 @@
         <v>82</v>
       </c>
       <c r="AF128" t="s" s="2">
-        <v>171</v>
+        <v>454</v>
       </c>
       <c r="AG128" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH128" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI128" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ128" t="s" s="2">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="AK128" t="s" s="2">
         <v>82</v>
@@ -18145,7 +18031,7 @@
         <v>82</v>
       </c>
       <c r="AM128" t="s" s="2">
-        <v>172</v>
+        <v>134</v>
       </c>
       <c r="AN128" t="s" s="2">
         <v>82</v>
@@ -18156,10 +18042,10 @@
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -18170,7 +18056,7 @@
         <v>80</v>
       </c>
       <c r="G129" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H129" t="s" s="2">
         <v>82</v>
@@ -18182,13 +18068,13 @@
         <v>82</v>
       </c>
       <c r="K129" t="s" s="2">
-        <v>136</v>
+        <v>702</v>
       </c>
       <c r="L129" t="s" s="2">
-        <v>137</v>
+        <v>776</v>
       </c>
       <c r="M129" t="s" s="2">
-        <v>138</v>
+        <v>777</v>
       </c>
       <c r="N129" s="2"/>
       <c r="O129" s="2"/>
@@ -18227,29 +18113,31 @@
         <v>82</v>
       </c>
       <c r="AB129" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AC129" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="AC129" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="AD129" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE129" t="s" s="2">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="AF129" t="s" s="2">
-        <v>176</v>
+        <v>775</v>
       </c>
       <c r="AG129" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH129" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI129" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ129" t="s" s="2">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="AK129" t="s" s="2">
         <v>82</v>
@@ -18258,7 +18146,7 @@
         <v>82</v>
       </c>
       <c r="AM129" t="s" s="2">
-        <v>82</v>
+        <v>778</v>
       </c>
       <c r="AN129" t="s" s="2">
         <v>82</v>
@@ -18269,14 +18157,12 @@
     </row>
     <row r="130">
       <c r="A130" t="s" s="2">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>782</v>
-      </c>
-      <c r="C130" t="s" s="2">
-        <v>784</v>
-      </c>
+        <v>779</v>
+      </c>
+      <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
         <v>82</v>
       </c>
@@ -18297,13 +18183,13 @@
         <v>82</v>
       </c>
       <c r="K130" t="s" s="2">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="L130" t="s" s="2">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="M130" t="s" s="2">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="N130" s="2"/>
       <c r="O130" s="2"/>
@@ -18354,19 +18240,19 @@
         <v>82</v>
       </c>
       <c r="AF130" t="s" s="2">
-        <v>176</v>
+        <v>779</v>
       </c>
       <c r="AG130" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH130" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI130" t="s" s="2">
-        <v>149</v>
+        <v>82</v>
       </c>
       <c r="AJ130" t="s" s="2">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="AK130" t="s" s="2">
         <v>82</v>
@@ -18375,7 +18261,7 @@
         <v>82</v>
       </c>
       <c r="AM130" t="s" s="2">
-        <v>82</v>
+        <v>783</v>
       </c>
       <c r="AN130" t="s" s="2">
         <v>82</v>
@@ -18386,14 +18272,12 @@
     </row>
     <row r="131">
       <c r="A131" t="s" s="2">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>782</v>
-      </c>
-      <c r="C131" t="s" s="2">
-        <v>789</v>
-      </c>
+        <v>784</v>
+      </c>
+      <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
         <v>82</v>
       </c>
@@ -18414,17 +18298,15 @@
         <v>82</v>
       </c>
       <c r="K131" t="s" s="2">
-        <v>790</v>
+        <v>780</v>
       </c>
       <c r="L131" t="s" s="2">
-        <v>791</v>
+        <v>785</v>
       </c>
       <c r="M131" t="s" s="2">
-        <v>792</v>
-      </c>
-      <c r="N131" t="s" s="2">
-        <v>793</v>
-      </c>
+        <v>786</v>
+      </c>
+      <c r="N131" s="2"/>
       <c r="O131" s="2"/>
       <c r="P131" t="s" s="2">
         <v>82</v>
@@ -18473,19 +18355,19 @@
         <v>82</v>
       </c>
       <c r="AF131" t="s" s="2">
-        <v>176</v>
+        <v>784</v>
       </c>
       <c r="AG131" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH131" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI131" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ131" t="s" s="2">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="AK131" t="s" s="2">
         <v>82</v>
@@ -18494,7 +18376,7 @@
         <v>82</v>
       </c>
       <c r="AM131" t="s" s="2">
-        <v>82</v>
+        <v>783</v>
       </c>
       <c r="AN131" t="s" s="2">
         <v>82</v>
@@ -18505,10 +18387,10 @@
     </row>
     <row r="132">
       <c r="A132" t="s" s="2">
-        <v>794</v>
+        <v>787</v>
       </c>
       <c r="B132" t="s" s="2">
-        <v>795</v>
+        <v>787</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
@@ -18531,16 +18413,20 @@
         <v>82</v>
       </c>
       <c r="K132" t="s" s="2">
-        <v>168</v>
+        <v>523</v>
       </c>
       <c r="L132" t="s" s="2">
-        <v>169</v>
+        <v>788</v>
       </c>
       <c r="M132" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="N132" s="2"/>
-      <c r="O132" s="2"/>
+        <v>789</v>
+      </c>
+      <c r="N132" t="s" s="2">
+        <v>790</v>
+      </c>
+      <c r="O132" t="s" s="2">
+        <v>791</v>
+      </c>
       <c r="P132" t="s" s="2">
         <v>82</v>
       </c>
@@ -18588,7 +18474,7 @@
         <v>82</v>
       </c>
       <c r="AF132" t="s" s="2">
-        <v>171</v>
+        <v>787</v>
       </c>
       <c r="AG132" t="s" s="2">
         <v>80</v>
@@ -18600,16 +18486,16 @@
         <v>82</v>
       </c>
       <c r="AJ132" t="s" s="2">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="AK132" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL132" t="s" s="2">
-        <v>82</v>
+        <v>792</v>
       </c>
       <c r="AM132" t="s" s="2">
-        <v>172</v>
+        <v>793</v>
       </c>
       <c r="AN132" t="s" s="2">
         <v>82</v>
@@ -18620,10 +18506,10 @@
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -18634,7 +18520,7 @@
         <v>80</v>
       </c>
       <c r="G133" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H133" t="s" s="2">
         <v>82</v>
@@ -18646,15 +18532,17 @@
         <v>82</v>
       </c>
       <c r="K133" t="s" s="2">
-        <v>136</v>
+        <v>621</v>
       </c>
       <c r="L133" t="s" s="2">
-        <v>137</v>
+        <v>795</v>
       </c>
       <c r="M133" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="N133" s="2"/>
+        <v>796</v>
+      </c>
+      <c r="N133" t="s" s="2">
+        <v>797</v>
+      </c>
       <c r="O133" s="2"/>
       <c r="P133" t="s" s="2">
         <v>82</v>
@@ -18691,54 +18579,54 @@
         <v>82</v>
       </c>
       <c r="AB133" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AC133" t="s" s="2">
-        <v>175</v>
+        <v>82</v>
       </c>
       <c r="AD133" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE133" t="s" s="2">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="AF133" t="s" s="2">
-        <v>176</v>
+        <v>794</v>
       </c>
       <c r="AG133" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH133" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI133" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ133" t="s" s="2">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="AK133" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL133" t="s" s="2">
-        <v>82</v>
+        <v>798</v>
       </c>
       <c r="AM133" t="s" s="2">
-        <v>82</v>
+        <v>799</v>
       </c>
       <c r="AN133" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO133" t="s" s="2">
-        <v>82</v>
+        <v>800</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s" s="2">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="B134" t="s" s="2">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="C134" s="2"/>
       <c r="D134" t="s" s="2">
@@ -18746,7 +18634,7 @@
       </c>
       <c r="E134" s="2"/>
       <c r="F134" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G134" t="s" s="2">
         <v>91</v>
@@ -18761,24 +18649,22 @@
         <v>82</v>
       </c>
       <c r="K134" t="s" s="2">
-        <v>105</v>
+        <v>702</v>
       </c>
       <c r="L134" t="s" s="2">
-        <v>185</v>
+        <v>802</v>
       </c>
       <c r="M134" t="s" s="2">
-        <v>186</v>
-      </c>
-      <c r="N134" t="s" s="2">
-        <v>187</v>
-      </c>
+        <v>803</v>
+      </c>
+      <c r="N134" s="2"/>
       <c r="O134" s="2"/>
       <c r="P134" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q134" s="2"/>
       <c r="R134" t="s" s="2">
-        <v>800</v>
+        <v>82</v>
       </c>
       <c r="S134" t="s" s="2">
         <v>82</v>
@@ -18820,10 +18706,10 @@
         <v>82</v>
       </c>
       <c r="AF134" t="s" s="2">
-        <v>188</v>
+        <v>801</v>
       </c>
       <c r="AG134" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AH134" t="s" s="2">
         <v>91</v>
@@ -18832,30 +18718,30 @@
         <v>82</v>
       </c>
       <c r="AJ134" t="s" s="2">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="AK134" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL134" t="s" s="2">
-        <v>82</v>
+        <v>804</v>
       </c>
       <c r="AM134" t="s" s="2">
-        <v>134</v>
+        <v>805</v>
       </c>
       <c r="AN134" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO134" t="s" s="2">
-        <v>82</v>
+        <v>806</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s" s="2">
-        <v>801</v>
+        <v>807</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>802</v>
+        <v>807</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -18863,7 +18749,7 @@
       </c>
       <c r="E135" s="2"/>
       <c r="F135" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G135" t="s" s="2">
         <v>91</v>
@@ -18878,15 +18764,17 @@
         <v>82</v>
       </c>
       <c r="K135" t="s" s="2">
-        <v>413</v>
+        <v>780</v>
       </c>
       <c r="L135" t="s" s="2">
-        <v>803</v>
+        <v>808</v>
       </c>
       <c r="M135" t="s" s="2">
-        <v>804</v>
-      </c>
-      <c r="N135" s="2"/>
+        <v>809</v>
+      </c>
+      <c r="N135" t="s" s="2">
+        <v>810</v>
+      </c>
       <c r="O135" s="2"/>
       <c r="P135" t="s" s="2">
         <v>82</v>
@@ -18935,7 +18823,7 @@
         <v>82</v>
       </c>
       <c r="AF135" t="s" s="2">
-        <v>194</v>
+        <v>807</v>
       </c>
       <c r="AG135" t="s" s="2">
         <v>80</v>
@@ -18953,10 +18841,10 @@
         <v>82</v>
       </c>
       <c r="AL135" t="s" s="2">
-        <v>82</v>
+        <v>811</v>
       </c>
       <c r="AM135" t="s" s="2">
-        <v>134</v>
+        <v>812</v>
       </c>
       <c r="AN135" t="s" s="2">
         <v>82</v>
@@ -18967,46 +18855,42 @@
     </row>
     <row r="136">
       <c r="A136" t="s" s="2">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="B136" t="s" s="2">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" t="s" s="2">
-        <v>451</v>
+        <v>82</v>
       </c>
       <c r="E136" s="2"/>
       <c r="F136" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G136" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H136" t="s" s="2">
         <v>82</v>
       </c>
       <c r="I136" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="J136" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="K136" t="s" s="2">
-        <v>136</v>
+        <v>814</v>
       </c>
       <c r="L136" t="s" s="2">
-        <v>452</v>
+        <v>815</v>
       </c>
       <c r="M136" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="N136" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="O136" t="s" s="2">
-        <v>220</v>
-      </c>
+        <v>816</v>
+      </c>
+      <c r="N136" s="2"/>
+      <c r="O136" s="2"/>
       <c r="P136" t="s" s="2">
         <v>82</v>
       </c>
@@ -19054,19 +18938,19 @@
         <v>82</v>
       </c>
       <c r="AF136" t="s" s="2">
-        <v>454</v>
+        <v>813</v>
       </c>
       <c r="AG136" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH136" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AI136" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ136" t="s" s="2">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="AK136" t="s" s="2">
         <v>82</v>
@@ -19075,10 +18959,10 @@
         <v>82</v>
       </c>
       <c r="AM136" t="s" s="2">
-        <v>134</v>
+        <v>817</v>
       </c>
       <c r="AN136" t="s" s="2">
-        <v>82</v>
+        <v>359</v>
       </c>
       <c r="AO136" t="s" s="2">
         <v>82</v>
@@ -19086,10 +18970,10 @@
     </row>
     <row r="137">
       <c r="A137" t="s" s="2">
-        <v>806</v>
+        <v>818</v>
       </c>
       <c r="B137" t="s" s="2">
-        <v>806</v>
+        <v>818</v>
       </c>
       <c r="C137" s="2"/>
       <c r="D137" t="s" s="2">
@@ -19112,17 +18996,15 @@
         <v>82</v>
       </c>
       <c r="K137" t="s" s="2">
-        <v>776</v>
+        <v>737</v>
       </c>
       <c r="L137" t="s" s="2">
-        <v>807</v>
+        <v>819</v>
       </c>
       <c r="M137" t="s" s="2">
-        <v>808</v>
-      </c>
-      <c r="N137" t="s" s="2">
-        <v>809</v>
-      </c>
+        <v>820</v>
+      </c>
+      <c r="N137" s="2"/>
       <c r="O137" s="2"/>
       <c r="P137" t="s" s="2">
         <v>82</v>
@@ -19171,7 +19053,7 @@
         <v>82</v>
       </c>
       <c r="AF137" t="s" s="2">
-        <v>806</v>
+        <v>818</v>
       </c>
       <c r="AG137" t="s" s="2">
         <v>80</v>
@@ -19189,10 +19071,10 @@
         <v>82</v>
       </c>
       <c r="AL137" t="s" s="2">
-        <v>82</v>
+        <v>821</v>
       </c>
       <c r="AM137" t="s" s="2">
-        <v>810</v>
+        <v>822</v>
       </c>
       <c r="AN137" t="s" s="2">
         <v>82</v>
@@ -19203,10 +19085,10 @@
     </row>
     <row r="138">
       <c r="A138" t="s" s="2">
-        <v>811</v>
+        <v>823</v>
       </c>
       <c r="B138" t="s" s="2">
-        <v>811</v>
+        <v>823</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" t="s" s="2">
@@ -19318,10 +19200,10 @@
     </row>
     <row r="139">
       <c r="A139" t="s" s="2">
-        <v>812</v>
+        <v>824</v>
       </c>
       <c r="B139" t="s" s="2">
-        <v>812</v>
+        <v>824</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" t="s" s="2">
@@ -19435,10 +19317,10 @@
     </row>
     <row r="140">
       <c r="A140" t="s" s="2">
-        <v>813</v>
+        <v>825</v>
       </c>
       <c r="B140" t="s" s="2">
-        <v>813</v>
+        <v>825</v>
       </c>
       <c r="C140" s="2"/>
       <c r="D140" t="s" s="2">
@@ -19554,10 +19436,10 @@
     </row>
     <row r="141">
       <c r="A141" t="s" s="2">
-        <v>814</v>
+        <v>826</v>
       </c>
       <c r="B141" t="s" s="2">
-        <v>814</v>
+        <v>826</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" t="s" s="2">
@@ -19565,7 +19447,7 @@
       </c>
       <c r="E141" s="2"/>
       <c r="F141" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G141" t="s" s="2">
         <v>91</v>
@@ -19580,15 +19462,17 @@
         <v>82</v>
       </c>
       <c r="K141" t="s" s="2">
-        <v>706</v>
+        <v>635</v>
       </c>
       <c r="L141" t="s" s="2">
-        <v>815</v>
+        <v>827</v>
       </c>
       <c r="M141" t="s" s="2">
-        <v>816</v>
-      </c>
-      <c r="N141" s="2"/>
+        <v>828</v>
+      </c>
+      <c r="N141" t="s" s="2">
+        <v>829</v>
+      </c>
       <c r="O141" s="2"/>
       <c r="P141" t="s" s="2">
         <v>82</v>
@@ -19613,34 +19497,32 @@
         <v>82</v>
       </c>
       <c r="X141" t="s" s="2">
-        <v>82</v>
+        <v>247</v>
       </c>
       <c r="Y141" t="s" s="2">
-        <v>82</v>
+        <v>830</v>
       </c>
       <c r="Z141" t="s" s="2">
-        <v>82</v>
+        <v>831</v>
       </c>
       <c r="AA141" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AB141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC141" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>518</v>
+      </c>
+      <c r="AC141" s="2"/>
       <c r="AD141" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE141" t="s" s="2">
-        <v>82</v>
+        <v>140</v>
       </c>
       <c r="AF141" t="s" s="2">
-        <v>814</v>
+        <v>826</v>
       </c>
       <c r="AG141" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AH141" t="s" s="2">
         <v>91</v>
@@ -19655,26 +19537,28 @@
         <v>82</v>
       </c>
       <c r="AL141" t="s" s="2">
-        <v>82</v>
+        <v>821</v>
       </c>
       <c r="AM141" t="s" s="2">
-        <v>817</v>
+        <v>832</v>
       </c>
       <c r="AN141" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO141" t="s" s="2">
-        <v>82</v>
+        <v>833</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s" s="2">
-        <v>818</v>
+        <v>834</v>
       </c>
       <c r="B142" t="s" s="2">
-        <v>818</v>
-      </c>
-      <c r="C142" s="2"/>
+        <v>826</v>
+      </c>
+      <c r="C142" t="s" s="2">
+        <v>835</v>
+      </c>
       <c r="D142" t="s" s="2">
         <v>82</v>
       </c>
@@ -19695,15 +19579,17 @@
         <v>82</v>
       </c>
       <c r="K142" t="s" s="2">
-        <v>819</v>
+        <v>201</v>
       </c>
       <c r="L142" t="s" s="2">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="M142" t="s" s="2">
-        <v>821</v>
-      </c>
-      <c r="N142" s="2"/>
+        <v>828</v>
+      </c>
+      <c r="N142" t="s" s="2">
+        <v>829</v>
+      </c>
       <c r="O142" s="2"/>
       <c r="P142" t="s" s="2">
         <v>82</v>
@@ -19728,13 +19614,11 @@
         <v>82</v>
       </c>
       <c r="X142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y142" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="Y142" s="2"/>
       <c r="Z142" t="s" s="2">
-        <v>82</v>
+        <v>836</v>
       </c>
       <c r="AA142" t="s" s="2">
         <v>82</v>
@@ -19752,10 +19636,10 @@
         <v>82</v>
       </c>
       <c r="AF142" t="s" s="2">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="AG142" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AH142" t="s" s="2">
         <v>91</v>
@@ -19770,24 +19654,24 @@
         <v>82</v>
       </c>
       <c r="AL142" t="s" s="2">
-        <v>82</v>
+        <v>821</v>
       </c>
       <c r="AM142" t="s" s="2">
-        <v>822</v>
+        <v>832</v>
       </c>
       <c r="AN142" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO142" t="s" s="2">
-        <v>82</v>
+        <v>833</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s" s="2">
-        <v>823</v>
+        <v>837</v>
       </c>
       <c r="B143" t="s" s="2">
-        <v>823</v>
+        <v>837</v>
       </c>
       <c r="C143" s="2"/>
       <c r="D143" t="s" s="2">
@@ -19810,13 +19694,13 @@
         <v>82</v>
       </c>
       <c r="K143" t="s" s="2">
-        <v>819</v>
+        <v>201</v>
       </c>
       <c r="L143" t="s" s="2">
-        <v>824</v>
+        <v>838</v>
       </c>
       <c r="M143" t="s" s="2">
-        <v>825</v>
+        <v>839</v>
       </c>
       <c r="N143" s="2"/>
       <c r="O143" s="2"/>
@@ -19843,13 +19727,13 @@
         <v>82</v>
       </c>
       <c r="X143" t="s" s="2">
-        <v>82</v>
+        <v>247</v>
       </c>
       <c r="Y143" t="s" s="2">
-        <v>82</v>
+        <v>840</v>
       </c>
       <c r="Z143" t="s" s="2">
-        <v>82</v>
+        <v>841</v>
       </c>
       <c r="AA143" t="s" s="2">
         <v>82</v>
@@ -19867,7 +19751,7 @@
         <v>82</v>
       </c>
       <c r="AF143" t="s" s="2">
-        <v>823</v>
+        <v>837</v>
       </c>
       <c r="AG143" t="s" s="2">
         <v>80</v>
@@ -19885,24 +19769,24 @@
         <v>82</v>
       </c>
       <c r="AL143" t="s" s="2">
-        <v>82</v>
+        <v>842</v>
       </c>
       <c r="AM143" t="s" s="2">
-        <v>822</v>
+        <v>843</v>
       </c>
       <c r="AN143" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO143" t="s" s="2">
-        <v>82</v>
+        <v>844</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s" s="2">
-        <v>826</v>
+        <v>845</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>826</v>
+        <v>845</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" t="s" s="2">
@@ -19925,20 +19809,16 @@
         <v>82</v>
       </c>
       <c r="K144" t="s" s="2">
-        <v>523</v>
+        <v>168</v>
       </c>
       <c r="L144" t="s" s="2">
-        <v>827</v>
+        <v>169</v>
       </c>
       <c r="M144" t="s" s="2">
-        <v>828</v>
-      </c>
-      <c r="N144" t="s" s="2">
-        <v>829</v>
-      </c>
-      <c r="O144" t="s" s="2">
-        <v>830</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="N144" s="2"/>
+      <c r="O144" s="2"/>
       <c r="P144" t="s" s="2">
         <v>82</v>
       </c>
@@ -19986,7 +19866,7 @@
         <v>82</v>
       </c>
       <c r="AF144" t="s" s="2">
-        <v>826</v>
+        <v>171</v>
       </c>
       <c r="AG144" t="s" s="2">
         <v>80</v>
@@ -19998,16 +19878,16 @@
         <v>82</v>
       </c>
       <c r="AJ144" t="s" s="2">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="AK144" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL144" t="s" s="2">
-        <v>831</v>
+        <v>82</v>
       </c>
       <c r="AM144" t="s" s="2">
-        <v>832</v>
+        <v>172</v>
       </c>
       <c r="AN144" t="s" s="2">
         <v>82</v>
@@ -20018,21 +19898,21 @@
     </row>
     <row r="145">
       <c r="A145" t="s" s="2">
-        <v>833</v>
+        <v>846</v>
       </c>
       <c r="B145" t="s" s="2">
-        <v>833</v>
+        <v>846</v>
       </c>
       <c r="C145" s="2"/>
       <c r="D145" t="s" s="2">
-        <v>82</v>
+        <v>216</v>
       </c>
       <c r="E145" s="2"/>
       <c r="F145" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G145" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H145" t="s" s="2">
         <v>82</v>
@@ -20044,16 +19924,16 @@
         <v>82</v>
       </c>
       <c r="K145" t="s" s="2">
-        <v>621</v>
+        <v>136</v>
       </c>
       <c r="L145" t="s" s="2">
-        <v>834</v>
+        <v>421</v>
       </c>
       <c r="M145" t="s" s="2">
-        <v>835</v>
+        <v>422</v>
       </c>
       <c r="N145" t="s" s="2">
-        <v>836</v>
+        <v>219</v>
       </c>
       <c r="O145" s="2"/>
       <c r="P145" t="s" s="2">
@@ -20091,54 +19971,54 @@
         <v>82</v>
       </c>
       <c r="AB145" t="s" s="2">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="AC145" t="s" s="2">
-        <v>82</v>
+        <v>175</v>
       </c>
       <c r="AD145" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE145" t="s" s="2">
-        <v>82</v>
+        <v>140</v>
       </c>
       <c r="AF145" t="s" s="2">
-        <v>833</v>
+        <v>176</v>
       </c>
       <c r="AG145" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH145" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI145" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ145" t="s" s="2">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="AK145" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AL145" t="s" s="2">
-        <v>837</v>
+        <v>82</v>
       </c>
       <c r="AM145" t="s" s="2">
-        <v>838</v>
+        <v>172</v>
       </c>
       <c r="AN145" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO145" t="s" s="2">
-        <v>839</v>
+        <v>82</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s" s="2">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="B146" t="s" s="2">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" t="s" s="2">
@@ -20149,7 +20029,7 @@
         <v>80</v>
       </c>
       <c r="G146" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H146" t="s" s="2">
         <v>82</v>
@@ -20158,19 +20038,23 @@
         <v>82</v>
       </c>
       <c r="J146" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K146" t="s" s="2">
-        <v>706</v>
+        <v>848</v>
       </c>
       <c r="L146" t="s" s="2">
-        <v>841</v>
+        <v>849</v>
       </c>
       <c r="M146" t="s" s="2">
-        <v>842</v>
-      </c>
-      <c r="N146" s="2"/>
-      <c r="O146" s="2"/>
+        <v>850</v>
+      </c>
+      <c r="N146" t="s" s="2">
+        <v>851</v>
+      </c>
+      <c r="O146" t="s" s="2">
+        <v>852</v>
+      </c>
       <c r="P146" t="s" s="2">
         <v>82</v>
       </c>
@@ -20218,13 +20102,13 @@
         <v>82</v>
       </c>
       <c r="AF146" t="s" s="2">
-        <v>840</v>
+        <v>853</v>
       </c>
       <c r="AG146" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH146" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI146" t="s" s="2">
         <v>82</v>
@@ -20236,24 +20120,24 @@
         <v>82</v>
       </c>
       <c r="AL146" t="s" s="2">
-        <v>843</v>
+        <v>82</v>
       </c>
       <c r="AM146" t="s" s="2">
-        <v>844</v>
+        <v>854</v>
       </c>
       <c r="AN146" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO146" t="s" s="2">
-        <v>845</v>
+        <v>855</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s" s="2">
-        <v>846</v>
+        <v>856</v>
       </c>
       <c r="B147" t="s" s="2">
-        <v>846</v>
+        <v>856</v>
       </c>
       <c r="C147" s="2"/>
       <c r="D147" t="s" s="2">
@@ -20273,21 +20157,23 @@
         <v>82</v>
       </c>
       <c r="J147" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="K147" t="s" s="2">
-        <v>819</v>
+        <v>168</v>
       </c>
       <c r="L147" t="s" s="2">
-        <v>847</v>
+        <v>857</v>
       </c>
       <c r="M147" t="s" s="2">
-        <v>848</v>
+        <v>858</v>
       </c>
       <c r="N147" t="s" s="2">
-        <v>849</v>
-      </c>
-      <c r="O147" s="2"/>
+        <v>859</v>
+      </c>
+      <c r="O147" t="s" s="2">
+        <v>860</v>
+      </c>
       <c r="P147" t="s" s="2">
         <v>82</v>
       </c>
@@ -20335,7 +20221,7 @@
         <v>82</v>
       </c>
       <c r="AF147" t="s" s="2">
-        <v>846</v>
+        <v>861</v>
       </c>
       <c r="AG147" t="s" s="2">
         <v>80</v>
@@ -20353,24 +20239,24 @@
         <v>82</v>
       </c>
       <c r="AL147" t="s" s="2">
-        <v>850</v>
+        <v>82</v>
       </c>
       <c r="AM147" t="s" s="2">
-        <v>851</v>
+        <v>862</v>
       </c>
       <c r="AN147" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO147" t="s" s="2">
-        <v>82</v>
+        <v>863</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s" s="2">
-        <v>852</v>
+        <v>864</v>
       </c>
       <c r="B148" t="s" s="2">
-        <v>852</v>
+        <v>864</v>
       </c>
       <c r="C148" s="2"/>
       <c r="D148" t="s" s="2">
@@ -20393,13 +20279,13 @@
         <v>82</v>
       </c>
       <c r="K148" t="s" s="2">
-        <v>853</v>
+        <v>865</v>
       </c>
       <c r="L148" t="s" s="2">
-        <v>854</v>
+        <v>866</v>
       </c>
       <c r="M148" t="s" s="2">
-        <v>855</v>
+        <v>867</v>
       </c>
       <c r="N148" s="2"/>
       <c r="O148" s="2"/>
@@ -20450,7 +20336,7 @@
         <v>82</v>
       </c>
       <c r="AF148" t="s" s="2">
-        <v>852</v>
+        <v>864</v>
       </c>
       <c r="AG148" t="s" s="2">
         <v>80</v>
@@ -20465,16 +20351,16 @@
         <v>103</v>
       </c>
       <c r="AK148" t="s" s="2">
-        <v>82</v>
+        <v>868</v>
       </c>
       <c r="AL148" t="s" s="2">
-        <v>82</v>
+        <v>842</v>
       </c>
       <c r="AM148" t="s" s="2">
-        <v>856</v>
+        <v>869</v>
       </c>
       <c r="AN148" t="s" s="2">
-        <v>359</v>
+        <v>82</v>
       </c>
       <c r="AO148" t="s" s="2">
         <v>82</v>
@@ -20482,21 +20368,21 @@
     </row>
     <row r="149">
       <c r="A149" t="s" s="2">
-        <v>857</v>
+        <v>870</v>
       </c>
       <c r="B149" t="s" s="2">
-        <v>857</v>
+        <v>870</v>
       </c>
       <c r="C149" s="2"/>
       <c r="D149" t="s" s="2">
-        <v>82</v>
+        <v>871</v>
       </c>
       <c r="E149" s="2"/>
       <c r="F149" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G149" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H149" t="s" s="2">
         <v>82</v>
@@ -20508,15 +20394,17 @@
         <v>82</v>
       </c>
       <c r="K149" t="s" s="2">
-        <v>776</v>
+        <v>872</v>
       </c>
       <c r="L149" t="s" s="2">
-        <v>858</v>
+        <v>873</v>
       </c>
       <c r="M149" t="s" s="2">
-        <v>859</v>
-      </c>
-      <c r="N149" s="2"/>
+        <v>874</v>
+      </c>
+      <c r="N149" t="s" s="2">
+        <v>875</v>
+      </c>
       <c r="O149" s="2"/>
       <c r="P149" t="s" s="2">
         <v>82</v>
@@ -20565,13 +20453,13 @@
         <v>82</v>
       </c>
       <c r="AF149" t="s" s="2">
-        <v>857</v>
+        <v>870</v>
       </c>
       <c r="AG149" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH149" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI149" t="s" s="2">
         <v>82</v>
@@ -20583,10 +20471,10 @@
         <v>82</v>
       </c>
       <c r="AL149" t="s" s="2">
-        <v>860</v>
+        <v>82</v>
       </c>
       <c r="AM149" t="s" s="2">
-        <v>861</v>
+        <v>876</v>
       </c>
       <c r="AN149" t="s" s="2">
         <v>82</v>
@@ -20597,10 +20485,10 @@
     </row>
     <row r="150">
       <c r="A150" t="s" s="2">
-        <v>862</v>
+        <v>877</v>
       </c>
       <c r="B150" t="s" s="2">
-        <v>862</v>
+        <v>877</v>
       </c>
       <c r="C150" s="2"/>
       <c r="D150" t="s" s="2">
@@ -20611,7 +20499,7 @@
         <v>80</v>
       </c>
       <c r="G150" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H150" t="s" s="2">
         <v>82</v>
@@ -20623,15 +20511,17 @@
         <v>82</v>
       </c>
       <c r="K150" t="s" s="2">
-        <v>168</v>
+        <v>878</v>
       </c>
       <c r="L150" t="s" s="2">
-        <v>169</v>
+        <v>879</v>
       </c>
       <c r="M150" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="N150" s="2"/>
+        <v>880</v>
+      </c>
+      <c r="N150" t="s" s="2">
+        <v>881</v>
+      </c>
       <c r="O150" s="2"/>
       <c r="P150" t="s" s="2">
         <v>82</v>
@@ -20680,1435 +20570,33 @@
         <v>82</v>
       </c>
       <c r="AF150" t="s" s="2">
-        <v>171</v>
+        <v>877</v>
       </c>
       <c r="AG150" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH150" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="AI150" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AJ150" t="s" s="2">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="AK150" t="s" s="2">
-        <v>82</v>
+        <v>882</v>
       </c>
       <c r="AL150" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AM150" t="s" s="2">
-        <v>172</v>
+        <v>883</v>
       </c>
       <c r="AN150" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AO150" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="s" s="2">
-        <v>863</v>
-      </c>
-      <c r="B151" t="s" s="2">
-        <v>863</v>
-      </c>
-      <c r="C151" s="2"/>
-      <c r="D151" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="E151" s="2"/>
-      <c r="F151" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G151" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K151" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="L151" t="s" s="2">
-        <v>421</v>
-      </c>
-      <c r="M151" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="N151" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="O151" s="2"/>
-      <c r="P151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q151" s="2"/>
-      <c r="R151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF151" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="AG151" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH151" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ151" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AK151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM151" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="AN151" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO151" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="s" s="2">
-        <v>864</v>
-      </c>
-      <c r="B152" t="s" s="2">
-        <v>864</v>
-      </c>
-      <c r="C152" s="2"/>
-      <c r="D152" t="s" s="2">
-        <v>451</v>
-      </c>
-      <c r="E152" s="2"/>
-      <c r="F152" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G152" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I152" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="J152" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K152" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="L152" t="s" s="2">
-        <v>452</v>
-      </c>
-      <c r="M152" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="N152" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="O152" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="P152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q152" s="2"/>
-      <c r="R152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF152" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="AG152" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH152" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ152" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AK152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM152" t="s" s="2">
-        <v>134</v>
-      </c>
-      <c r="AN152" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO152" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="B153" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="C153" s="2"/>
-      <c r="D153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E153" s="2"/>
-      <c r="F153" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="G153" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K153" t="s" s="2">
-        <v>635</v>
-      </c>
-      <c r="L153" t="s" s="2">
-        <v>866</v>
-      </c>
-      <c r="M153" t="s" s="2">
-        <v>867</v>
-      </c>
-      <c r="N153" t="s" s="2">
-        <v>868</v>
-      </c>
-      <c r="O153" s="2"/>
-      <c r="P153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q153" s="2"/>
-      <c r="R153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X153" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="Y153" t="s" s="2">
-        <v>869</v>
-      </c>
-      <c r="Z153" t="s" s="2">
-        <v>870</v>
-      </c>
-      <c r="AA153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB153" t="s" s="2">
-        <v>518</v>
-      </c>
-      <c r="AC153" s="2"/>
-      <c r="AD153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE153" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="AF153" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="AG153" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AH153" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ153" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL153" t="s" s="2">
-        <v>860</v>
-      </c>
-      <c r="AM153" t="s" s="2">
-        <v>871</v>
-      </c>
-      <c r="AN153" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO153" t="s" s="2">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="s" s="2">
-        <v>873</v>
-      </c>
-      <c r="B154" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="C154" t="s" s="2">
-        <v>874</v>
-      </c>
-      <c r="D154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E154" s="2"/>
-      <c r="F154" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G154" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K154" t="s" s="2">
-        <v>201</v>
-      </c>
-      <c r="L154" t="s" s="2">
-        <v>866</v>
-      </c>
-      <c r="M154" t="s" s="2">
-        <v>867</v>
-      </c>
-      <c r="N154" t="s" s="2">
-        <v>868</v>
-      </c>
-      <c r="O154" s="2"/>
-      <c r="P154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q154" s="2"/>
-      <c r="R154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X154" t="s" s="2">
-        <v>236</v>
-      </c>
-      <c r="Y154" s="2"/>
-      <c r="Z154" t="s" s="2">
-        <v>875</v>
-      </c>
-      <c r="AA154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF154" t="s" s="2">
-        <v>865</v>
-      </c>
-      <c r="AG154" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AH154" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ154" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL154" t="s" s="2">
-        <v>860</v>
-      </c>
-      <c r="AM154" t="s" s="2">
-        <v>871</v>
-      </c>
-      <c r="AN154" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO154" t="s" s="2">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="s" s="2">
-        <v>876</v>
-      </c>
-      <c r="B155" t="s" s="2">
-        <v>876</v>
-      </c>
-      <c r="C155" s="2"/>
-      <c r="D155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E155" s="2"/>
-      <c r="F155" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G155" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K155" t="s" s="2">
-        <v>201</v>
-      </c>
-      <c r="L155" t="s" s="2">
-        <v>877</v>
-      </c>
-      <c r="M155" t="s" s="2">
-        <v>878</v>
-      </c>
-      <c r="N155" s="2"/>
-      <c r="O155" s="2"/>
-      <c r="P155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q155" s="2"/>
-      <c r="R155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X155" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="Y155" t="s" s="2">
-        <v>879</v>
-      </c>
-      <c r="Z155" t="s" s="2">
-        <v>880</v>
-      </c>
-      <c r="AA155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF155" t="s" s="2">
-        <v>876</v>
-      </c>
-      <c r="AG155" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH155" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ155" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL155" t="s" s="2">
-        <v>881</v>
-      </c>
-      <c r="AM155" t="s" s="2">
-        <v>882</v>
-      </c>
-      <c r="AN155" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO155" t="s" s="2">
-        <v>883</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="s" s="2">
-        <v>884</v>
-      </c>
-      <c r="B156" t="s" s="2">
-        <v>884</v>
-      </c>
-      <c r="C156" s="2"/>
-      <c r="D156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E156" s="2"/>
-      <c r="F156" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G156" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K156" t="s" s="2">
-        <v>168</v>
-      </c>
-      <c r="L156" t="s" s="2">
-        <v>169</v>
-      </c>
-      <c r="M156" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="N156" s="2"/>
-      <c r="O156" s="2"/>
-      <c r="P156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q156" s="2"/>
-      <c r="R156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF156" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="AG156" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH156" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM156" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="AN156" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO156" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="s" s="2">
-        <v>885</v>
-      </c>
-      <c r="B157" t="s" s="2">
-        <v>885</v>
-      </c>
-      <c r="C157" s="2"/>
-      <c r="D157" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="E157" s="2"/>
-      <c r="F157" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G157" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K157" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="L157" t="s" s="2">
-        <v>421</v>
-      </c>
-      <c r="M157" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="N157" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="O157" s="2"/>
-      <c r="P157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q157" s="2"/>
-      <c r="R157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB157" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AC157" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="AD157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE157" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="AF157" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="AG157" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH157" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ157" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AK157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM157" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="AN157" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO157" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="s" s="2">
-        <v>886</v>
-      </c>
-      <c r="B158" t="s" s="2">
-        <v>886</v>
-      </c>
-      <c r="C158" s="2"/>
-      <c r="D158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E158" s="2"/>
-      <c r="F158" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G158" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J158" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K158" t="s" s="2">
-        <v>887</v>
-      </c>
-      <c r="L158" t="s" s="2">
-        <v>888</v>
-      </c>
-      <c r="M158" t="s" s="2">
-        <v>889</v>
-      </c>
-      <c r="N158" t="s" s="2">
-        <v>890</v>
-      </c>
-      <c r="O158" t="s" s="2">
-        <v>891</v>
-      </c>
-      <c r="P158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q158" s="2"/>
-      <c r="R158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF158" t="s" s="2">
-        <v>892</v>
-      </c>
-      <c r="AG158" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH158" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ158" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM158" t="s" s="2">
-        <v>893</v>
-      </c>
-      <c r="AN158" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO158" t="s" s="2">
-        <v>894</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="s" s="2">
-        <v>895</v>
-      </c>
-      <c r="B159" t="s" s="2">
-        <v>895</v>
-      </c>
-      <c r="C159" s="2"/>
-      <c r="D159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E159" s="2"/>
-      <c r="F159" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G159" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J159" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K159" t="s" s="2">
-        <v>168</v>
-      </c>
-      <c r="L159" t="s" s="2">
-        <v>896</v>
-      </c>
-      <c r="M159" t="s" s="2">
-        <v>897</v>
-      </c>
-      <c r="N159" t="s" s="2">
-        <v>898</v>
-      </c>
-      <c r="O159" t="s" s="2">
-        <v>899</v>
-      </c>
-      <c r="P159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q159" s="2"/>
-      <c r="R159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF159" t="s" s="2">
-        <v>900</v>
-      </c>
-      <c r="AG159" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH159" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ159" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM159" t="s" s="2">
-        <v>901</v>
-      </c>
-      <c r="AN159" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO159" t="s" s="2">
-        <v>902</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="s" s="2">
-        <v>903</v>
-      </c>
-      <c r="B160" t="s" s="2">
-        <v>903</v>
-      </c>
-      <c r="C160" s="2"/>
-      <c r="D160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E160" s="2"/>
-      <c r="F160" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G160" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K160" t="s" s="2">
-        <v>904</v>
-      </c>
-      <c r="L160" t="s" s="2">
-        <v>905</v>
-      </c>
-      <c r="M160" t="s" s="2">
-        <v>906</v>
-      </c>
-      <c r="N160" s="2"/>
-      <c r="O160" s="2"/>
-      <c r="P160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q160" s="2"/>
-      <c r="R160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF160" t="s" s="2">
-        <v>903</v>
-      </c>
-      <c r="AG160" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH160" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ160" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK160" t="s" s="2">
-        <v>907</v>
-      </c>
-      <c r="AL160" t="s" s="2">
-        <v>881</v>
-      </c>
-      <c r="AM160" t="s" s="2">
-        <v>908</v>
-      </c>
-      <c r="AN160" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO160" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="s" s="2">
-        <v>909</v>
-      </c>
-      <c r="B161" t="s" s="2">
-        <v>909</v>
-      </c>
-      <c r="C161" s="2"/>
-      <c r="D161" t="s" s="2">
-        <v>910</v>
-      </c>
-      <c r="E161" s="2"/>
-      <c r="F161" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G161" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K161" t="s" s="2">
-        <v>911</v>
-      </c>
-      <c r="L161" t="s" s="2">
-        <v>912</v>
-      </c>
-      <c r="M161" t="s" s="2">
-        <v>913</v>
-      </c>
-      <c r="N161" t="s" s="2">
-        <v>914</v>
-      </c>
-      <c r="O161" s="2"/>
-      <c r="P161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q161" s="2"/>
-      <c r="R161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF161" t="s" s="2">
-        <v>909</v>
-      </c>
-      <c r="AG161" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH161" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ161" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM161" t="s" s="2">
-        <v>915</v>
-      </c>
-      <c r="AN161" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO161" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="s" s="2">
-        <v>916</v>
-      </c>
-      <c r="B162" t="s" s="2">
-        <v>916</v>
-      </c>
-      <c r="C162" s="2"/>
-      <c r="D162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E162" s="2"/>
-      <c r="F162" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G162" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K162" t="s" s="2">
-        <v>917</v>
-      </c>
-      <c r="L162" t="s" s="2">
-        <v>918</v>
-      </c>
-      <c r="M162" t="s" s="2">
-        <v>919</v>
-      </c>
-      <c r="N162" t="s" s="2">
-        <v>920</v>
-      </c>
-      <c r="O162" s="2"/>
-      <c r="P162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q162" s="2"/>
-      <c r="R162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF162" t="s" s="2">
-        <v>916</v>
-      </c>
-      <c r="AG162" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH162" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ162" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AK162" t="s" s="2">
-        <v>921</v>
-      </c>
-      <c r="AL162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM162" t="s" s="2">
-        <v>922</v>
-      </c>
-      <c r="AN162" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO162" t="s" s="2">
         <v>82</v>
       </c>
     </row>

</xml_diff>